<commit_message>
feat: update Feishu material intake workflow
</commit_message>
<xml_diff>
--- a/案例素材清单.xlsx
+++ b/案例素材清单.xlsx
@@ -1191,7 +1191,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1249,6 +1249,53 @@
       <c r="I1" s="3" t="inlineStr">
         <is>
           <t>存放文件夹</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>西湖_湖面风景背景图.jpg</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>西湖风景</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>西湖湖面远景实拍，湖水、远山、天空与岸边枝叶构成宁静开阔的自然画面</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>封面页背景 / 章节过渡页 / 氛围底图</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>西湖自然风光，天高云淡、湖面开阔，适合作为方案封面、章节页或过渡页的氛围背景素材</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>自有，需确认</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>已识别</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>背景素材_氛围图</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: restore docs and revert generated material lists
</commit_message>
<xml_diff>
--- a/案例素材清单.xlsx
+++ b/案例素材清单.xlsx
@@ -1191,7 +1191,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1252,53 +1252,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>西湖_湖面风景背景图.jpg</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>西湖风景</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>西湖湖面远景实拍，湖水、远山、天空与岸边枝叶构成宁静开阔的自然画面</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>封面页背景 / 章节过渡页 / 氛围底图</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>西湖自然风光，天高云淡、湖面开阔，适合作为方案封面、章节页或过渡页的氛围背景素材</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>无</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>自有，需确认</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>已识别</t>
-        </is>
-      </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>背景素材_氛围图</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>